<commit_message>
Add dynamic coating support from Excel
</commit_message>
<xml_diff>
--- a/prices.xlsx
+++ b/prices.xlsx
@@ -397,13 +397,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:F20"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
     <col min="3" max="3" width="10.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="25.83203125" customWidth="1"/>
     <col min="5" max="5" width="12.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -417,9 +418,12 @@
         <v>thickness</v>
       </c>
       <c r="D1" t="str">
+        <v>coating</v>
+      </c>
+      <c r="E1" t="str">
         <v>color</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>price</v>
       </c>
     </row>
@@ -431,13 +435,16 @@
         <v>S-8</v>
       </c>
       <c r="C2" t="str">
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="D2" t="str">
-        <v/>
-      </c>
-      <c r="E2">
-        <v>580</v>
+        <v>Эконом Полиэстер</v>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2">
+        <v>545</v>
       </c>
     </row>
     <row r="3">
@@ -451,10 +458,13 @@
         <v>0.45</v>
       </c>
       <c r="D3" t="str">
-        <v/>
-      </c>
-      <c r="E3">
-        <v>650</v>
+        <v>Стандарт Полиэстер</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Цинк</v>
+      </c>
+      <c r="F3">
+        <v>575</v>
       </c>
     </row>
     <row r="4">
@@ -468,10 +478,13 @@
         <v>0.45</v>
       </c>
       <c r="D4" t="str">
-        <v>Цинк</v>
-      </c>
-      <c r="E4">
-        <v>610</v>
+        <v>Стандарт Полиэстер</v>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4">
+        <v>585</v>
       </c>
     </row>
     <row r="5">
@@ -482,13 +495,16 @@
         <v>S-8</v>
       </c>
       <c r="C5" t="str">
-        <v>0.5</v>
+        <v>0.45</v>
       </c>
       <c r="D5" t="str">
-        <v/>
-      </c>
-      <c r="E5">
-        <v>720</v>
+        <v>Стальной бархат</v>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5">
+        <v>870</v>
       </c>
     </row>
     <row r="6">
@@ -499,13 +515,16 @@
         <v>S-8</v>
       </c>
       <c r="C6" t="str">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="D6" t="str">
-        <v/>
-      </c>
-      <c r="E6">
-        <v>890</v>
+        <v>Printech</v>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6">
+        <v>1375</v>
       </c>
     </row>
     <row r="7">
@@ -513,16 +532,19 @@
         <v>profnastil</v>
       </c>
       <c r="B7" t="str">
-        <v>NS-10</v>
+        <v>S-8</v>
       </c>
       <c r="C7" t="str">
-        <v>0.35</v>
+        <v>0.5</v>
       </c>
       <c r="D7" t="str">
-        <v/>
-      </c>
-      <c r="E7">
-        <v>590</v>
+        <v>Стандарт Полиэстер</v>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7">
+        <v>719</v>
       </c>
     </row>
     <row r="8">
@@ -530,143 +552,167 @@
         <v>profnastil</v>
       </c>
       <c r="B8" t="str">
-        <v>NS-10</v>
+        <v>S-8</v>
       </c>
       <c r="C8" t="str">
-        <v>0.45</v>
+        <v>0.5</v>
       </c>
       <c r="D8" t="str">
-        <v/>
-      </c>
-      <c r="E8">
-        <v>660</v>
+        <v>High Gloss Matt</v>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8">
+        <v>1133</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>profnastil</v>
+        <v>metallocherepica</v>
       </c>
       <c r="B9" t="str">
-        <v>NS-10</v>
+        <v>monterej</v>
       </c>
       <c r="C9" t="str">
-        <v>0.5</v>
+        <v>0.45</v>
       </c>
       <c r="D9" t="str">
-        <v/>
-      </c>
-      <c r="E9">
-        <v>730</v>
+        <v>Стандарт Полиэстер</v>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9">
+        <v>720</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>profnastil</v>
+        <v>metallocherepica</v>
       </c>
       <c r="B10" t="str">
-        <v>NS-10</v>
+        <v>monterej</v>
       </c>
       <c r="C10" t="str">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="D10" t="str">
-        <v/>
-      </c>
-      <c r="E10">
-        <v>900</v>
+        <v>Стальной бархат</v>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+      <c r="F10">
+        <v>950</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>profnastil</v>
+        <v>saiding</v>
       </c>
       <c r="B11" t="str">
-        <v>NS-20</v>
+        <v>korabelnaya</v>
       </c>
       <c r="C11" t="str">
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="D11" t="str">
-        <v/>
-      </c>
-      <c r="E11">
-        <v>600</v>
+        <v>Стандарт Полиэстер</v>
+      </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
+      <c r="F11">
+        <v>760</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>profnastil</v>
+        <v>saiding</v>
       </c>
       <c r="B12" t="str">
-        <v>NS-20</v>
+        <v>korabelnaya</v>
       </c>
       <c r="C12" t="str">
         <v>0.45</v>
       </c>
       <c r="D12" t="str">
-        <v/>
-      </c>
-      <c r="E12">
-        <v>670</v>
+        <v>Printech</v>
+      </c>
+      <c r="E12" t="str">
+        <v/>
+      </c>
+      <c r="F12">
+        <v>1400</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>profnastil</v>
+        <v>shtaketnik</v>
       </c>
       <c r="B13" t="str">
-        <v>NS-20</v>
+        <v>uzkiy</v>
       </c>
       <c r="C13" t="str">
-        <v>0.5</v>
+        <v>0.45</v>
       </c>
       <c r="D13" t="str">
         <v/>
       </c>
-      <c r="E13">
-        <v>740</v>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+      <c r="F13">
+        <v>500</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>profnastil</v>
+        <v>shtaketnik</v>
       </c>
       <c r="B14" t="str">
-        <v>NS-20</v>
+        <v>polukrugly</v>
       </c>
       <c r="C14" t="str">
-        <v>0.65</v>
+        <v>0.45</v>
       </c>
       <c r="D14" t="str">
         <v/>
       </c>
-      <c r="E14">
-        <v>910</v>
+      <c r="E14" t="str">
+        <v/>
+      </c>
+      <c r="F14">
+        <v>520</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>profnastil</v>
+        <v>shtaketnik</v>
       </c>
       <c r="B15" t="str">
-        <v>S-21</v>
+        <v>figurny</v>
       </c>
       <c r="C15" t="str">
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="D15" t="str">
         <v/>
       </c>
-      <c r="E15">
-        <v>610</v>
+      <c r="E15" t="str">
+        <v/>
+      </c>
+      <c r="F15">
+        <v>530</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>profnastil</v>
+        <v>shtaketnik</v>
       </c>
       <c r="B16" t="str">
-        <v>S-21</v>
+        <v>shirokiy</v>
       </c>
       <c r="C16" t="str">
         <v>0.45</v>
@@ -674,33 +720,39 @@
       <c r="D16" t="str">
         <v/>
       </c>
-      <c r="E16">
-        <v>680</v>
+      <c r="E16" t="str">
+        <v/>
+      </c>
+      <c r="F16">
+        <v>540</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>profnastil</v>
+        <v>shtaketnik</v>
       </c>
       <c r="B17" t="str">
-        <v>S-21</v>
+        <v>pletenka</v>
       </c>
       <c r="C17" t="str">
-        <v>0.5</v>
+        <v>0.45</v>
       </c>
       <c r="D17" t="str">
         <v/>
       </c>
-      <c r="E17">
-        <v>750</v>
+      <c r="E17" t="str">
+        <v/>
+      </c>
+      <c r="F17">
+        <v>560</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>profnastil</v>
+        <v>lameli</v>
       </c>
       <c r="B18" t="str">
-        <v>NS-21</v>
+        <v>evrozhaluzi</v>
       </c>
       <c r="C18" t="str">
         <v>0.45</v>
@@ -708,16 +760,19 @@
       <c r="D18" t="str">
         <v/>
       </c>
-      <c r="E18">
-        <v>690</v>
+      <c r="E18" t="str">
+        <v/>
+      </c>
+      <c r="F18">
+        <v>850</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>profnastil</v>
+        <v>dobornie</v>
       </c>
       <c r="B19" t="str">
-        <v>NS-35</v>
+        <v>individual</v>
       </c>
       <c r="C19" t="str">
         <v>0.45</v>
@@ -725,302 +780,36 @@
       <c r="D19" t="str">
         <v/>
       </c>
-      <c r="E19">
-        <v>710</v>
+      <c r="E19" t="str">
+        <v/>
+      </c>
+      <c r="F19">
+        <v>700</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>profnastil</v>
+        <v>dobornie</v>
       </c>
       <c r="B20" t="str">
-        <v>S-44</v>
+        <v>individual</v>
       </c>
       <c r="C20" t="str">
-        <v>0.45</v>
+        <v>0.5</v>
       </c>
       <c r="D20" t="str">
         <v/>
       </c>
-      <c r="E20">
-        <v>730</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>profnastil</v>
-      </c>
-      <c r="B21" t="str">
-        <v>N-60</v>
-      </c>
-      <c r="C21" t="str">
-        <v>0.45</v>
-      </c>
-      <c r="D21" t="str">
-        <v/>
-      </c>
-      <c r="E21">
-        <v>760</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>profnastil</v>
-      </c>
-      <c r="B22" t="str">
-        <v>N-75</v>
-      </c>
-      <c r="C22" t="str">
-        <v>0.45</v>
-      </c>
-      <c r="D22" t="str">
-        <v/>
-      </c>
-      <c r="E22">
-        <v>790</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v>metallocherepica</v>
-      </c>
-      <c r="B23" t="str">
-        <v>monterej</v>
-      </c>
-      <c r="C23" t="str">
-        <v>0.45</v>
-      </c>
-      <c r="D23" t="str">
-        <v/>
-      </c>
-      <c r="E23">
-        <v>720</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="str">
-        <v>metallocherepica</v>
-      </c>
-      <c r="B24" t="str">
-        <v>monterej</v>
-      </c>
-      <c r="C24" t="str">
-        <v>0.5</v>
-      </c>
-      <c r="D24" t="str">
-        <v/>
-      </c>
-      <c r="E24">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v>saiding</v>
-      </c>
-      <c r="B25" t="str">
-        <v>korabelnaya</v>
-      </c>
-      <c r="C25" t="str">
-        <v>0.45</v>
-      </c>
-      <c r="D25" t="str">
-        <v/>
-      </c>
-      <c r="E25">
-        <v>760</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="str">
-        <v>saiding</v>
-      </c>
-      <c r="B26" t="str">
-        <v>evrobrus</v>
-      </c>
-      <c r="C26" t="str">
-        <v>0.45</v>
-      </c>
-      <c r="D26" t="str">
-        <v/>
-      </c>
-      <c r="E26">
-        <v>770</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="str">
-        <v>saiding</v>
-      </c>
-      <c r="B27" t="str">
-        <v>blokkhaus</v>
-      </c>
-      <c r="C27" t="str">
-        <v>0.45</v>
-      </c>
-      <c r="D27" t="str">
-        <v/>
-      </c>
-      <c r="E27">
-        <v>780</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="str">
-        <v>saiding</v>
-      </c>
-      <c r="B28" t="str">
-        <v>brevno4d</v>
-      </c>
-      <c r="C28" t="str">
-        <v>0.45</v>
-      </c>
-      <c r="D28" t="str">
-        <v/>
-      </c>
-      <c r="E28">
-        <v>790</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="str">
-        <v>shtaketnik</v>
-      </c>
-      <c r="B29" t="str">
-        <v>uzkiy</v>
-      </c>
-      <c r="C29" t="str">
-        <v>0.45</v>
-      </c>
-      <c r="D29" t="str">
-        <v/>
-      </c>
-      <c r="E29">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="str">
-        <v>shtaketnik</v>
-      </c>
-      <c r="B30" t="str">
-        <v>polukrugly</v>
-      </c>
-      <c r="C30" t="str">
-        <v>0.45</v>
-      </c>
-      <c r="D30" t="str">
-        <v/>
-      </c>
-      <c r="E30">
-        <v>520</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="str">
-        <v>shtaketnik</v>
-      </c>
-      <c r="B31" t="str">
-        <v>figurny</v>
-      </c>
-      <c r="C31" t="str">
-        <v>0.45</v>
-      </c>
-      <c r="D31" t="str">
-        <v/>
-      </c>
-      <c r="E31">
-        <v>530</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="str">
-        <v>shtaketnik</v>
-      </c>
-      <c r="B32" t="str">
-        <v>shirokiy</v>
-      </c>
-      <c r="C32" t="str">
-        <v>0.45</v>
-      </c>
-      <c r="D32" t="str">
-        <v/>
-      </c>
-      <c r="E32">
-        <v>540</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="str">
-        <v>shtaketnik</v>
-      </c>
-      <c r="B33" t="str">
-        <v>pletenka</v>
-      </c>
-      <c r="C33" t="str">
-        <v>0.45</v>
-      </c>
-      <c r="D33" t="str">
-        <v/>
-      </c>
-      <c r="E33">
-        <v>560</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="str">
-        <v>lameli</v>
-      </c>
-      <c r="B34" t="str">
-        <v>evrozhaluzi</v>
-      </c>
-      <c r="C34" t="str">
-        <v>0.45</v>
-      </c>
-      <c r="D34" t="str">
-        <v/>
-      </c>
-      <c r="E34">
-        <v>850</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="str">
-        <v>dobornie</v>
-      </c>
-      <c r="B35" t="str">
-        <v>individual</v>
-      </c>
-      <c r="C35" t="str">
-        <v>0.45</v>
-      </c>
-      <c r="D35" t="str">
-        <v/>
-      </c>
-      <c r="E35">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="str">
-        <v>dobornie</v>
-      </c>
-      <c r="B36" t="str">
-        <v>individual</v>
-      </c>
-      <c r="C36" t="str">
-        <v>0.5</v>
-      </c>
-      <c r="D36" t="str">
-        <v/>
-      </c>
-      <c r="E36">
+      <c r="E20" t="str">
+        <v/>
+      </c>
+      <c r="F20">
         <v>770</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E36"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F20"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>